<commit_message>
Update beta dataset after Swisscom quality sprint
</commit_message>
<xml_diff>
--- a/exports/swiss_equity_data_public_beta.xlsx
+++ b/exports/swiss_equity_data_public_beta.xlsx
@@ -4025,7 +4025,9 @@
       <c r="I36" t="n">
         <v>4293</v>
       </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="n">
+        <v>2148</v>
+      </c>
       <c r="K36" t="n">
         <v>1604</v>
       </c>
@@ -4062,12 +4064,12 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>6/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>10/13</t>
+          <t>12/13</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -4221,7 +4223,9 @@
       <c r="I38" t="n">
         <v>4213</v>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="n">
+        <v>2069</v>
+      </c>
       <c r="K38" t="n">
         <v>1521</v>
       </c>
@@ -4260,12 +4264,12 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>6/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>13/13</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -4529,7 +4533,9 @@
       <c r="L41" t="n">
         <v>35.37</v>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="n">
+        <v>24801</v>
+      </c>
       <c r="N41" t="n">
         <v>10813</v>
       </c>
@@ -4554,15 +4560,17 @@
       <c r="U41" t="n">
         <v>22</v>
       </c>
-      <c r="V41" t="inlineStr"/>
+      <c r="V41" t="n">
+        <v>43.6</v>
+      </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>6/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>12/13</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -4626,7 +4634,9 @@
       <c r="L42" t="n">
         <v>30.93</v>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="n">
+        <v>24620</v>
+      </c>
       <c r="N42" t="n">
         <v>11171</v>
       </c>
@@ -4651,15 +4661,17 @@
       <c r="U42" t="n">
         <v>22</v>
       </c>
-      <c r="V42" t="inlineStr"/>
+      <c r="V42" t="n">
+        <v>45.37</v>
+      </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>6/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>12/13</t>
+          <t>13/13</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
@@ -4822,8 +4834,12 @@
       <c r="L44" t="n">
         <v>29.77</v>
       </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>37211</v>
+      </c>
+      <c r="N44" t="n">
+        <v>12155</v>
+      </c>
       <c r="O44" t="n">
         <v>17535</v>
       </c>
@@ -4845,20 +4861,22 @@
       <c r="U44" t="n">
         <v>22</v>
       </c>
-      <c r="V44" t="inlineStr"/>
+      <c r="V44" t="n">
+        <v>32.67</v>
+      </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>5/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>13/13</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="Z44" t="inlineStr">
@@ -8927,14 +8945,18 @@
       <c r="N36" t="n">
         <v>5.5</v>
       </c>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" t="n">
+        <v>11</v>
+      </c>
       <c r="P36" t="n">
         <v>11.8</v>
       </c>
       <c r="Q36" t="n">
         <v>7.39</v>
       </c>
-      <c r="R36" t="inlineStr"/>
+      <c r="R36" t="n">
+        <v>18.44885338830198</v>
+      </c>
       <c r="S36" t="n">
         <v>36.87194022159238</v>
       </c>
@@ -9083,14 +9105,18 @@
       <c r="N38" t="n">
         <v>6.2</v>
       </c>
-      <c r="O38" t="inlineStr"/>
+      <c r="O38" t="n">
+        <v>12.6</v>
+      </c>
       <c r="P38" t="n">
         <v>13.3</v>
       </c>
       <c r="Q38" t="n">
         <v>6.52</v>
       </c>
-      <c r="R38" t="inlineStr"/>
+      <c r="R38" t="n">
+        <v>17.66262591770531</v>
+      </c>
       <c r="S38" t="n">
         <v>35.96551135393546</v>
       </c>
@@ -9537,9 +9563,15 @@
       <c r="H44" t="n">
         <v>15.6</v>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
+      <c r="I44" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="J44" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1.44</v>
+      </c>
       <c r="L44" t="n">
         <v>19058</v>
       </c>
@@ -12172,22 +12204,22 @@
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations.</t>
+          <t>Some values are calculated or have acceptable limitations.</t>
         </is>
       </c>
     </row>
@@ -12262,22 +12294,22 @@
         <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations.</t>
+          <t>Some values are calculated or have acceptable limitations.</t>
         </is>
       </c>
     </row>
@@ -12397,22 +12429,22 @@
         <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations. Some values are calculated rather than directly reported.</t>
+          <t>Some values are calculated or have acceptable limitations. Some values are calculated rather than directly reported.</t>
         </is>
       </c>
     </row>
@@ -12442,22 +12474,22 @@
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations.</t>
+          <t>Some values are calculated or have acceptable limitations.</t>
         </is>
       </c>
     </row>
@@ -12532,22 +12564,22 @@
         <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations.</t>
+          <t>Some values are calculated or have acceptable limitations.</t>
         </is>
       </c>
     </row>
@@ -13102,7 +13134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15115,33 +15147,33 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>missing_capex</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>ebit</t>
+          <t>capex_m</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>capex_m absent — FCF proxy unavailable</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>The field 'ebit' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
         </is>
       </c>
     </row>
@@ -15162,7 +15194,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -15213,22 +15245,24 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>missing_capex</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>capex_m</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>-474</v>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>capex_m absent — FCF proxy unavailable</t>
+          <t>cash_m = -474.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -15243,7 +15277,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
@@ -15264,37 +15298,39 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>ebit</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
+          <t>free_cash_flow_final_m</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1543</v>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>FCF = op_cf - abs(capex) = 1543.0 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>The field 'ebit' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
@@ -15315,7 +15351,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -15328,11 +15364,11 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>-474</v>
+        <v>-328</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>cash_m = -474.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>cash_m = -328.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -15368,7 +15404,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -15381,11 +15417,11 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1543</v>
+        <v>1840</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = 1543.0 CHF M; not reported by company</t>
+          <t>FCF = op_cf - abs(capex) = 1840.0 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -15421,7 +15457,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -15434,11 +15470,11 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>-328</v>
+        <v>-340</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>cash_m = -328.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>cash_m = -340.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -15474,7 +15510,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -15487,11 +15523,11 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>1840</v>
+        <v>1758</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = 1840.0 CHF M; not reported by company</t>
+          <t>FCF = op_cf - abs(capex) = 1758.0 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -15527,7 +15563,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -15540,11 +15576,11 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>-340</v>
+        <v>-401</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>cash_m = -340.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>cash_m = -401.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -15580,39 +15616,39 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
+          <t>cash_m</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>1758</v>
+        <v>-121</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = 1758.0 CHF M; not reported by company</t>
+          <t>cash_m = -121.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
@@ -15633,37 +15669,39 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>total_assets</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>-148</v>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>cash_m = -148.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>The field 'total_assets' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
@@ -15684,7 +15722,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -15697,11 +15735,11 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>-401</v>
+        <v>-1523</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>cash_m = -401.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>cash_m = -1523.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -15737,283 +15775,283 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>total_assets</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr"/>
+          <t>free_cash_flow_final_m</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>2285</v>
+      </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>FCF = op_cf - abs(capex) = 2285.0 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>The field 'total_assets' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>per_share_not_comparable_pre_split</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>-121</v>
-      </c>
+          <t>pe_ratio,dividend_yield_pct</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>cash_m = -121.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2023</v>
+        <v>2016</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>per_share_not_comparable_pre_split</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>-148</v>
-      </c>
+          <t>pe_ratio,dividend_yield_pct</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>cash_m = -148.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2024</v>
+        <v>2017</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>per_share_not_comparable_pre_split</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>total_assets</t>
+          <t>pe_ratio,dividend_yield_pct</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>The field 'total_assets' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2024</v>
+        <v>2018</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>free_cash_flow_implausible</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>total_equity</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr"/>
+          <t>free_cash_flow</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>38.8</v>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>FCF (38.8) differs by &gt;50% from op_cf-abs(capex) (510.6).</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>The field 'total_equity' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2024</v>
+        <v>2018</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>price_to_fcf_extreme</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>cash_m</t>
+          <t>price_to_fcf</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>-1523</v>
+        <v>458.9</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>cash_m = -1523.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>Price/FCF is 458.9, absolute value &gt; 200.</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -16028,60 +16066,60 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>The price-to-free-cash-flow ratio is unusually large for this year, typically because free cash flow was near zero or very small relative to market cap. Treat this ratio with caution.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>free_cash_flow_implausible</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
+          <t>free_cash_flow</t>
         </is>
       </c>
       <c r="G57" t="n">
-        <v>2285</v>
+        <v>-717</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = 2285.0 CHF M; not reported by company</t>
+          <t>FCF (-717.0) differs by &gt;50% from op_cf-abs(capex) (1034.2).</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
+          <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
         </is>
       </c>
     </row>
@@ -16102,349 +16140,37 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>per_share_not_comparable_pre_split</t>
+          <t>free_cash_flow_implausible</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>pe_ratio,dividend_yield_pct</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr"/>
+          <t>free_cash_flow</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>-1870.1</v>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
+          <t>FCF (-1870.1) differs by &gt;50% from op_cf-abs(capex) (1388.6).</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
-        <is>
-          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>2016</v>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>per_share_not_comparable_pre_split</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>pe_ratio,dividend_yield_pct</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>Informational note</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>2017</v>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>per_share_not_comparable_pre_split</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>pe_ratio,dividend_yield_pct</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>Informational note</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>2018</v>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>free_cash_flow_implausible</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>38.8</v>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>FCF (38.8) differs by &gt;50% from op_cf-abs(capex) (510.6).</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
-        <v>2018</v>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>price_to_fcf_extreme</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>price_to_fcf</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>458.9</v>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Price/FCF is 458.9, absolute value &gt; 200.</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>The price-to-free-cash-flow ratio is unusually large for this year, typically because free cash flow was near zero or very small relative to market cap. Treat this ratio with caution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>2019</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>free_cash_flow_implausible</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>-717</v>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>FCF (-717.0) differs by &gt;50% from op_cf-abs(capex) (1034.2).</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>free_cash_flow_implausible</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G64" t="n">
-        <v>-1870.1</v>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>FCF (-1870.1) differs by &gt;50% from op_cf-abs(capex) (1388.6).</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
         <is>
           <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
         </is>

</xml_diff>

<commit_message>
Finalize beta dataset quality layer
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/swiss_equity_data_public_beta.xlsx
+++ b/exports/swiss_equity_data_public_beta.xlsx
@@ -653,21 +653,29 @@
       <c r="M2" t="n">
         <v>4095.8</v>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>1539.7</v>
+      </c>
       <c r="O2" t="n">
         <v>102.6</v>
       </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="n">
+        <v>244.9</v>
+      </c>
       <c r="S2" t="n">
         <v>-39.3</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>190.8</v>
+      </c>
       <c r="U2" t="n">
         <v>1.302</v>
       </c>
-      <c r="V2" t="inlineStr"/>
+      <c r="V2" t="n">
+        <v>37.59</v>
+      </c>
       <c r="W2" t="inlineStr">
         <is>
           <t>4/7</t>
@@ -680,7 +688,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -742,21 +750,29 @@
       <c r="M3" t="n">
         <v>4415.3</v>
       </c>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>1677.7</v>
+      </c>
       <c r="O3" t="n">
         <v>98.8</v>
       </c>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="n">
+        <v>166.4</v>
+      </c>
       <c r="S3" t="n">
         <v>-32.2</v>
       </c>
-      <c r="T3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>128.8</v>
+      </c>
       <c r="U3" t="n">
         <v>1.502</v>
       </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="V3" t="n">
+        <v>38</v>
+      </c>
       <c r="W3" t="inlineStr">
         <is>
           <t>4/7</t>
@@ -769,7 +785,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -932,7 +948,9 @@
       <c r="M5" t="n">
         <v>4895.4</v>
       </c>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="n">
+        <v>1768.6</v>
+      </c>
       <c r="O5" t="n">
         <v>140.5</v>
       </c>
@@ -950,7 +968,9 @@
       <c r="U5" t="n">
         <v>1.852</v>
       </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="V5" t="n">
+        <v>36.13</v>
+      </c>
       <c r="W5" t="inlineStr">
         <is>
           <t>5/7</t>
@@ -963,7 +983,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -1025,7 +1045,9 @@
       <c r="M6" t="n">
         <v>5353</v>
       </c>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>1834.6</v>
+      </c>
       <c r="O6" t="n">
         <v>279.7</v>
       </c>
@@ -1047,7 +1069,9 @@
       <c r="U6" t="n">
         <v>1.902</v>
       </c>
-      <c r="V6" t="inlineStr"/>
+      <c r="V6" t="n">
+        <v>34.27</v>
+      </c>
       <c r="W6" t="inlineStr">
         <is>
           <t>6/7</t>
@@ -1749,7 +1773,9 @@
       <c r="T13" t="n">
         <v>484</v>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="n">
+        <v>8.4</v>
+      </c>
       <c r="V13" t="n">
         <v>41.71</v>
       </c>
@@ -3262,7 +3288,9 @@
       <c r="T28" t="n">
         <v>-93.294</v>
       </c>
-      <c r="U28" t="inlineStr"/>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
       <c r="V28" t="n">
         <v>41.27</v>
       </c>
@@ -6311,7 +6339,9 @@
       <c r="T2" t="n">
         <v>1.98591156922832</v>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>1.898356349743304</v>
+      </c>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
@@ -6369,7 +6399,9 @@
       <c r="T3" t="n">
         <v>2.027567300003807</v>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>1.226059475307467</v>
+      </c>
       <c r="V3" t="n">
         <v>4.521033151589937</v>
       </c>
@@ -10671,25 +10703,25 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations.</t>
+          <t>No issues detected.</t>
         </is>
       </c>
     </row>
@@ -10716,25 +10748,25 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations.</t>
+          <t>No issues detected.</t>
         </is>
       </c>
     </row>
@@ -10809,22 +10841,22 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated rather than directly reported.</t>
+          <t>Some values are calculated rather than directly reported.</t>
         </is>
       </c>
     </row>
@@ -10854,22 +10886,22 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency.</t>
+          <t>No issues detected.</t>
         </is>
       </c>
     </row>
@@ -11166,7 +11198,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -11175,7 +11207,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -11841,7 +11873,7 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -11850,7 +11882,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -11889,22 +11921,22 @@
         <v>2</v>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations.</t>
+          <t>Some values are calculated or have acceptable limitations.</t>
         </is>
       </c>
     </row>
@@ -12024,22 +12056,22 @@
         <v>2</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Usable with notes</t>
+          <t>High confidence</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Some fields are missing and flagged for transparency. Some values are calculated or have acceptable limitations.</t>
+          <t>Some values are calculated or have acceptable limitations.</t>
         </is>
       </c>
     </row>
@@ -13134,7 +13166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13224,37 +13256,39 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>free_cash_flow_final_m</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>144.6</v>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>FCF = op_cf - abs(capex) = 144.6 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The field 'free_cash_flow' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
@@ -13275,37 +13309,39 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>total_equity</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>-680.8</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>cash_m = -680.8 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>The field 'total_equity' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
@@ -13326,37 +13362,39 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2015</v>
+        <v>2021</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>operating_cash_flow_missing</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>operating_cash_flow</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>-673.7</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Operating cash flow is missing.</t>
+          <t>cash_m = -673.7 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Operating cash flow was not extracted for this company and year.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
@@ -13377,22 +13415,24 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>missing_free_cash_flow_final</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>-636.4</v>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m absent — no reported FCF and op_cf/capex unavailable</t>
+          <t>cash_m = -636.4 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -13407,7 +13447,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Free cash flow is unavailable for this year because neither a reported figure nor the required inputs (operating cash flow and capex) could be extracted.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
@@ -13428,37 +13468,39 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2016</v>
+        <v>2023</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>-687.2</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>cash_m = -687.2 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>The field 'free_cash_flow' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
@@ -13479,37 +13521,39 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2016</v>
+        <v>2024</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>total_equity</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>-609.1</v>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>cash_m = -609.1 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>The field 'total_equity' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
@@ -13530,73 +13574,75 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2016</v>
+        <v>2025</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>operating_cash_flow_missing</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>operating_cash_flow</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>-538.4</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Operating cash flow is missing.</t>
+          <t>cash_m = -538.4 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Operating cash flow was not extracted for this company and year.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>GEBN.SW</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>Geberit AG</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>missing_free_cash_flow_final</t>
+          <t>missing_dividend_yield</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
+          <t>dividend_yield_pct</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m absent — no reported FCF and op_cf/capex unavailable</t>
+          <t>dividend_yield_pct unavailable — dividend_per_share absent</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -13611,28 +13657,28 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Free cash flow is unavailable for this year because neither a reported figure nor the required inputs (operating cash flow and capex) could be extracted.</t>
+          <t>Dividend yield could not be calculated because dividend per share is not available for this year.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -13645,11 +13691,11 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>144.6</v>
+        <v>-34.029</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = 144.6 CHF M; not reported by company</t>
+          <t>FCF = op_cf - abs(capex) = -34.029 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -13671,246 +13717,248 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>total_equity</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>free_cash_flow_final_m</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>-41.941</v>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>FCF = op_cf - abs(capex) = -41.941 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>The field 'total_equity' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>total_equity</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>free_cash_flow_final_m</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>-37.57</v>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>FCF = op_cf - abs(capex) = -37.57 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>The field 'total_equity' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>cash_m</t>
+          <t>free_cash_flow_final_m</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>-680.8</v>
+        <v>-139.673</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>cash_m = -680.8 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>FCF = op_cf - abs(capex) = -139.673 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>cash_m</t>
+          <t>free_cash_flow_final_m</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>-673.7</v>
+        <v>-93.294</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>cash_m = -673.7 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>FCF = op_cf - abs(capex) = -93.294 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>missing_dividend_yield</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>-636.4</v>
-      </c>
+          <t>dividend_yield_pct</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>cash_m = -636.4 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>dividend_yield_pct unavailable — dividend_per_share absent</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -13925,45 +13973,43 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>Dividend yield could not be calculated because dividend per share is not available for this year.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>missing_capex</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>-687.2</v>
-      </c>
+          <t>capex_m</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>cash_m = -687.2 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>capex_m absent — FCF proxy unavailable</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -13978,45 +14024,43 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>missing_free_cash_flow_final</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>-609.1</v>
-      </c>
+          <t>free_cash_flow_final_m</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>cash_m = -609.1 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>Free cash flow is unavailable; HIAG does not report a direct FCF metric for this year.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -14031,147 +14075,149 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>HIAG does not report a direct free cash flow metric for this year, and no safe real-estate-specific methodology is documented. The field is left blank as a documented limitation.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DKSH.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DKSH Holding AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Distribution / Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>cash_m</t>
+          <t>free_cash_flow_final_m</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>-538.4</v>
+        <v>-76.20399999999999</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>cash_m = -538.4 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>FCF = op_cf - abs(capex) = -76.204 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GEBN.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Geberit AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>missing_dividend_per_share</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dividend_per_share</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>free_cash_flow_final_m</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>-71.22</v>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>dividend_per_share absent — dividend yield will be None</t>
+          <t>FCF = op_cf - abs(capex) = -71.22 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Dividend per share was not found in the annual report for this year.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GEBN.SW</t>
+          <t>HIAG.SW</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Geberit AG</t>
+          <t>HIAG Immobilien Holding AG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>missing_dividend_yield</t>
+          <t>missing_capex</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>dividend_yield_pct</t>
+          <t>capex_m</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>dividend_yield_pct unavailable — dividend_per_share absent</t>
+          <t>capex_m absent — FCF proxy unavailable</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -14186,7 +14232,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Dividend yield could not be calculated because dividend per share is not available for this year.</t>
+          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
         </is>
       </c>
     </row>
@@ -14207,11 +14253,11 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>missing_free_cash_flow_final</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -14219,27 +14265,25 @@
           <t>free_cash_flow_final_m</t>
         </is>
       </c>
-      <c r="G21" t="n">
-        <v>-34.029</v>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = -34.029 CHF M; not reported by company</t>
+          <t>Free cash flow is unavailable; HIAG does not report a direct FCF metric for this year.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
+          <t>HIAG does not report a direct free cash flow metric for this year, and no safe real-estate-specific methodology is documented. The field is left blank as a documented limitation.</t>
         </is>
       </c>
     </row>
@@ -14260,7 +14304,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2016</v>
+        <v>2024</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -14273,11 +14317,11 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>-41.941</v>
+        <v>21.085</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = -41.941 CHF M; not reported by company</t>
+          <t>FCF = op_cf - abs(capex) = 21.085 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -14313,7 +14357,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2017</v>
+        <v>2025</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -14326,11 +14370,11 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>-37.57</v>
+        <v>-88.515</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = -37.57 CHF M; not reported by company</t>
+          <t>FCF = op_cf - abs(capex) = -88.515 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -14352,142 +14396,138 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>missing_capex</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>-139.673</v>
-      </c>
+          <t>capex_m</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = -139.673 CHF M; not reported by company</t>
+          <t>capex_m absent — FCF proxy unavailable</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
+          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>missing_capex</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>-93.294</v>
-      </c>
+          <t>capex_m</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = -93.294 CHF M; not reported by company</t>
+          <t>capex_m absent — FCF proxy unavailable</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
+          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>missing_dividend_per_share</t>
+          <t>missing_capex</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dividend_per_share</t>
+          <t>capex_m</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>dividend_per_share absent — dividend yield will be None</t>
+          <t>capex_m absent — FCF proxy unavailable</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -14502,43 +14542,45 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Dividend per share was not found in the annual report for this year.</t>
+          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>missing_dividend_yield</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>dividend_yield_pct</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>-474</v>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>dividend_yield_pct unavailable — dividend_per_share absent</t>
+          <t>cash_m = -474.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -14553,94 +14595,98 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Dividend yield could not be calculated because dividend per share is not available for this year.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>free_cash_flow_final_m</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1543</v>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>FCF = op_cf - abs(capex) = 1543.0 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>The field 'free_cash_flow' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>missing_capex</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>capex_m</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>-328</v>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>capex_m absent — FCF proxy unavailable</t>
+          <t>cash_m = -328.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -14655,24 +14701,24 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -14680,7 +14726,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>missing_free_cash_flow_final</t>
+          <t>free_cash_flow_calculated</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -14688,99 +14734,101 @@
           <t>free_cash_flow_final_m</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>1840</v>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m absent — no reported FCF and op_cf/capex unavailable</t>
+          <t>FCF = op_cf - abs(capex) = 1840.0 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Free cash flow is unavailable for this year because neither a reported figure nor the required inputs (operating cash flow and capex) could be extracted.</t>
+          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
+          <t>cash_m</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>-76.20399999999999</v>
+        <v>-340</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = -76.204 CHF M; not reported by company</t>
+          <t>cash_m = -340.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -14793,11 +14841,11 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>-71.22</v>
+        <v>1758</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = -71.22 CHF M; not reported by company</t>
+          <t>FCF = op_cf - abs(capex) = 1758.0 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -14819,87 +14867,91 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>missing_public_field</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>-401</v>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Public beta field is missing in financials.csv.</t>
+          <t>cash_m = -401.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Needs review</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>The field 'free_cash_flow' is currently missing for this company and year. It could not be extracted from the annual report.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>missing_capex</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>capex_m</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>-121</v>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>capex_m absent — FCF proxy unavailable</t>
+          <t>cash_m = -121.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -14914,24 +14966,24 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -14939,18 +14991,20 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>missing_free_cash_flow_final</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr"/>
+          <t>cash_m</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>-148</v>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m absent — no reported FCF and op_cf/capex unavailable</t>
+          <t>cash_m = -148.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -14965,24 +15019,24 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Free cash flow is unavailable for this year because neither a reported figure nor the required inputs (operating cash flow and capex) could be extracted.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -14990,52 +15044,52 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>negative_cash</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
+          <t>cash_m</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>21.085</v>
+        <v>-1523</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = 21.085 CHF M; not reported by company</t>
+          <t>cash_m = -1523.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
+          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HIAG.SW</t>
+          <t>SCMN.SW</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>HIAG Immobilien Holding AG</t>
+          <t>Swisscom AG</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Telecom / Infrastructure</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -15052,11 +15106,11 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>-88.515</v>
+        <v>2285</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = -88.515 CHF M; not reported by company</t>
+          <t>FCF = op_cf - abs(capex) = 2285.0 CHF M; not reported by company</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -15078,17 +15132,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -15096,50 +15150,50 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>missing_capex</t>
+          <t>per_share_not_comparable_pre_split</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>capex_m</t>
+          <t>pe_ratio,dividend_yield_pct</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>capex_m absent — FCF proxy unavailable</t>
+          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
+          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -15147,50 +15201,50 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>missing_capex</t>
+          <t>per_share_not_comparable_pre_split</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>capex_m</t>
+          <t>pe_ratio,dividend_yield_pct</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>capex_m absent — FCF proxy unavailable</t>
+          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
+          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -15198,50 +15252,50 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>missing_capex</t>
+          <t>per_share_not_comparable_pre_split</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>capex_m</t>
+          <t>pe_ratio,dividend_yield_pct</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>capex_m absent — FCF proxy unavailable</t>
+          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Acceptable limitation</t>
+          <t>Informational note</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Capital expenditure was not extracted for this year. Free cash flow calculation from operating cash flow is therefore unavailable.</t>
+          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -15249,20 +15303,20 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>free_cash_flow_implausible</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>cash_m</t>
+          <t>free_cash_flow</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>-474</v>
+        <v>38.8</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>cash_m = -474.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>FCF (38.8) differs by &gt;50% from op_cf-abs(capex) (510.6).</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -15277,77 +15331,77 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>price_to_fcf_extreme</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
+          <t>price_to_fcf</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>1543</v>
+        <v>458.9</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = 1543.0 CHF M; not reported by company</t>
+          <t>Price/FCF is 458.9, absolute value &gt; 200.</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
+          <t>The price-to-free-cash-flow ratio is unusually large for this year, typically because free cash flow was near zero or very small relative to market cap. Treat this ratio with caution.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -15355,20 +15409,20 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>negative_cash</t>
+          <t>free_cash_flow_implausible</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>cash_m</t>
+          <t>free_cash_flow</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>-328</v>
+        <v>-717</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>cash_m = -328.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
+          <t>FCF (-717.0) differs by &gt;50% from op_cf-abs(capex) (1034.2).</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -15383,794 +15437,58 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
+          <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SCMN.SW</t>
+          <t>SIKA.SW</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Swisscom AG</t>
+          <t>Sika AG</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Telecom / Infrastructure</t>
+          <t>Chemicals / Construction Materials</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>free_cash_flow_calculated</t>
+          <t>free_cash_flow_implausible</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>free_cash_flow_final_m</t>
+          <t>free_cash_flow</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1840</v>
+        <v>-1870.1</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>FCF = op_cf - abs(capex) = 1840.0 CHF M; not reported by company</t>
+          <t>FCF (-1870.1) differs by &gt;50% from op_cf-abs(capex) (1388.6).</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Informational note</t>
+          <t>Acceptable limitation</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
-        <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>SCMN.SW</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Swisscom AG</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Telecom / Infrastructure</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>2020</v>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>negative_cash</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>-340</v>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>cash_m = -340.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>SCMN.SW</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Swisscom AG</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Telecom / Infrastructure</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>2021</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>free_cash_flow_calculated</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>free_cash_flow_final_m</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>1758</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>FCF = op_cf - abs(capex) = 1758.0 CHF M; not reported by company</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>Informational note</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>SCMN.SW</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Swisscom AG</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Telecom / Infrastructure</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>2021</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>negative_cash</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>-401</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>cash_m = -401.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>SCMN.SW</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Swisscom AG</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Telecom / Infrastructure</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>2022</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>negative_cash</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>-121</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>cash_m = -121.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>SCMN.SW</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Swisscom AG</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Telecom / Infrastructure</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>negative_cash</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>-148</v>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>cash_m = -148.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>SCMN.SW</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Swisscom AG</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Telecom / Infrastructure</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>2024</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>negative_cash</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>cash_m</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>-1523</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>cash_m = -1523.0 CHF M — likely overdraft netting in source report; used as-is in EV / net_debt calculations</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Cash is reported as a negative value and is used as-is. This typically occurs due to overdraft netting or cash pooling presentation in the annual report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>SCMN.SW</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Swisscom AG</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Telecom / Infrastructure</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>2025</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>free_cash_flow_calculated</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>free_cash_flow_final_m</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>2285</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>FCF = op_cf - abs(capex) = 2285.0 CHF M; not reported by company</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Informational note</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Free cash flow was not reported directly by the company. It has been calculated as operating cash flow minus capital expenditure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>2015</v>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>per_share_not_comparable_pre_split</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>pe_ratio,dividend_yield_pct</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Informational note</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>2016</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>per_share_not_comparable_pre_split</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>pe_ratio,dividend_yield_pct</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Informational note</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>2017</v>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>per_share_not_comparable_pre_split</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>pe_ratio,dividend_yield_pct</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Sika 2015-2017 EPS/DPS are pre-split registered-share values and are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Informational note</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>P/E ratio and dividend yield are intentionally blank for these years. Pre-split per-share figures are not comparable with split-adjusted market prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>2018</v>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>free_cash_flow_implausible</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>38.8</v>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>FCF (38.8) differs by &gt;50% from op_cf-abs(capex) (510.6).</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>2018</v>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>price_to_fcf_extreme</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>price_to_fcf</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>458.9</v>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Price/FCF is 458.9, absolute value &gt; 200.</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>The price-to-free-cash-flow ratio is unusually large for this year, typically because free cash flow was near zero or very small relative to market cap. Treat this ratio with caution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>2019</v>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>free_cash_flow_implausible</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>-717</v>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>FCF (-717.0) differs by &gt;50% from op_cf-abs(capex) (1034.2).</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>SIKA.SW</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Sika AG</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Chemicals / Construction Materials</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>free_cash_flow_implausible</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>free_cash_flow</t>
-        </is>
-      </c>
-      <c r="G58" t="n">
-        <v>-1870.1</v>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>FCF (-1870.1) differs by &gt;50% from op_cf-abs(capex) (1388.6).</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Acceptable limitation</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
         <is>
           <t>The reported or calculated free cash flow appears implausibly small relative to operating cash flow and capital expenditure.</t>
         </is>

</xml_diff>